<commit_message>
Function names are updates
</commit_message>
<xml_diff>
--- a/InterfaceProject/filtered_scenarios_Carla.xlsx
+++ b/InterfaceProject/filtered_scenarios_Carla.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AL37"/>
+  <dimension ref="A1:AL23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -622,21 +622,21 @@
     </row>
     <row r="2">
       <c r="A2" t="n">
-        <v>7</v>
+        <v>3</v>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>SC2-S13</t>
+          <t>SC2-S8</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Ego vehicle approaching slower lead vehicle</t>
+          <t xml:space="preserve"> Lead vehicle braking</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>Another vehicle is driving in front of the ego vehicle at a slower speed. As a result, the other vehicle appears in the ego vehicle’s f ield of view. The ego vehicle might brake to avoid a collision.</t>
+          <t>The ego vehicle is following another vehicle. The other vehicle is referred to as the lead vehicle. The lead vehicle brakes, such that the ego vehicle has to adapt its speed in order to stay at a safe distance from the lead vehicle.</t>
         </is>
       </c>
       <c r="E2" t="n">
@@ -658,10 +658,10 @@
         <v>0</v>
       </c>
       <c r="K2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="L2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="M2" t="n">
         <v>0</v>
@@ -724,17 +724,17 @@
         <v>0</v>
       </c>
       <c r="AG2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AH2" t="n">
         <v>0</v>
       </c>
       <c r="AI2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AJ2" t="inlineStr">
         <is>
-          <t>sc13.png</t>
+          <t>sc8.png</t>
         </is>
       </c>
       <c r="AK2" t="inlineStr">
@@ -750,21 +750,21 @@
     </row>
     <row r="3">
       <c r="A3" t="n">
-        <v>8</v>
+        <v>20</v>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>SC2-S14</t>
+          <t>SC2-S65</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Ego vehicle approaching stopped lead vehicle</t>
+          <t>Turning lead vehicle</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>A lead vehicle driving in front of the ego vehicle at a slower speed . The reason for the other vehicle to come to a full stop is, e.g., because of a traffic light. The objective of the ego vehicle is to continue driving in the same direction.</t>
+          <t xml:space="preserve">The ego vehicle is approaching a junction while following its lead vehicle. The ego vehicle intends to go straight at the junction while the preceding vehicle turns left or right at the junction. </t>
         </is>
       </c>
       <c r="E3" t="n">
@@ -786,10 +786,10 @@
         <v>0</v>
       </c>
       <c r="K3" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="L3" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="M3" t="n">
         <v>0</v>
@@ -855,14 +855,14 @@
         <v>0</v>
       </c>
       <c r="AH3" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AI3" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AJ3" t="inlineStr">
         <is>
-          <t>sc14.png</t>
+          <t>sc65.png</t>
         </is>
       </c>
       <c r="AK3" t="inlineStr">
@@ -878,22 +878,21 @@
     </row>
     <row r="4">
       <c r="A4" t="n">
-        <v>21</v>
+        <v>9</v>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>SC2-S31</t>
+          <t>SC2-S27</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Ego straight with vehicle from left at non-signalized
- junction</t>
+          <t>Ego vehicle turns right at signalized junction</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t xml:space="preserve">The ego vehicle is approaching a junction that is not equipped with traffic light signals. The objective of the ego vehicle is to go straight at the junction. Another vehicle is approaching the junction from the left side of the ego vehicle. The direction of the other vehicle is not further specified. </t>
+          <t>The ego vehicle is approaching a junction that is equipped with traffic light signals. The ego vehicle intends to turn right and other vehicle is going straight.</t>
         </is>
       </c>
       <c r="E4" t="n">
@@ -981,17 +980,17 @@
         <v>0</v>
       </c>
       <c r="AG4" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AH4" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AI4" t="n">
         <v>0</v>
       </c>
       <c r="AJ4" t="inlineStr">
         <is>
-          <t>sc31.png</t>
+          <t>sc261.png</t>
         </is>
       </c>
       <c r="AK4" t="inlineStr">
@@ -1007,21 +1006,21 @@
     </row>
     <row r="5">
       <c r="A5" t="n">
-        <v>25</v>
+        <v>11</v>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>SC2-S36</t>
+          <t>SC2-S29</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Undertaking at left turn at non-signalized junction</t>
+          <t>Oncomingvehicle turns right at non-signalized junction</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t xml:space="preserve">The ego vehicle is approaching a junction that is not equipped with traffic light signals. The ego vehicle intends to turn left at the junction. Another vehicle is driving in the same direction in the left lane next to the ego vehicle. </t>
+          <t>The ego vehicle is approaching a junction that is not equipped with traffic light signals. It intended direction of the ego vehicle is not specified. Another vehicle is approaching the junction from the opposite direction. The other vehicle intends to turn right at the junction, such that the trajectories of the other vehicle and the ego vehicle might intersect</t>
         </is>
       </c>
       <c r="E5" t="n">
@@ -1119,7 +1118,7 @@
       </c>
       <c r="AJ5" t="inlineStr">
         <is>
-          <t>sc36.png</t>
+          <t>sc29.png</t>
         </is>
       </c>
       <c r="AK5" t="inlineStr">
@@ -1135,22 +1134,22 @@
     </row>
     <row r="6">
       <c r="A6" t="n">
-        <v>24</v>
+        <v>13</v>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>SC2-S35</t>
+          <t>SC2-S31</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t xml:space="preserve"> Ego and crossing vehicle turn right at non-signalized
+          <t>Ego straight with vehicle from left at non-signalized
  junction</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>The ego vehicle is approaching a junction that is not equipped with traffic light signals. The ego vehicle intends to turn right at the junction. Another vehicle is approaching the junction from the left or right side of the ego vehicle. The other vehicle also turns right at the junction, such that the trajectories of the ego vehicle and the other vehicle intersect.</t>
+          <t xml:space="preserve">The ego vehicle is approaching a junction that is not equipped with traffic light signals. The objective of the ego vehicle is to go straight at the junction. Another vehicle is approaching the junction from the left side of the ego vehicle. The direction of the other vehicle is not further specified. </t>
         </is>
       </c>
       <c r="E6" t="n">
@@ -1248,7 +1247,7 @@
       </c>
       <c r="AJ6" t="inlineStr">
         <is>
-          <t>sc35.png</t>
+          <t>sc31.png</t>
         </is>
       </c>
       <c r="AK6" t="inlineStr">
@@ -1264,22 +1263,22 @@
     </row>
     <row r="7">
       <c r="A7" t="n">
-        <v>23</v>
+        <v>14</v>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>SC2-S34</t>
+          <t>SC2-S32</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>Ego vehicle turns right and ends up in same direction
- as other vehicle at non-signalized junction</t>
+          <t xml:space="preserve"> Vehicle straight with ego from left at non-signalized
+ junction</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t xml:space="preserve">The ego vehicle is approaching a junction that is not equipped with traffic light signals. The ego vehicle intends to turn right at the junction. Another vehicle is approaching the junction from the left side of the ego vehicle. The other vehicle goes straight at the junction, such that it ends up in the same direction as the ego vehicle. </t>
+          <t>The ego vehicle is approaching a junc tion that is not equipped with traffic light signals. Another vehicle is also approaching the junction and its trajectory intersects the ego vehicle’s trajectory. The other vehicle is ap proaching the junction from the right side of the ego vehicle and this vehicle goes straight at the junction.</t>
         </is>
       </c>
       <c r="E7" t="n">
@@ -1301,13 +1300,13 @@
         <v>0</v>
       </c>
       <c r="K7" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="L7" t="n">
         <v>0</v>
       </c>
       <c r="M7" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="N7" t="n">
         <v>0</v>
@@ -1322,7 +1321,7 @@
         <v>0</v>
       </c>
       <c r="R7" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="S7" t="n">
         <v>0</v>
@@ -1343,7 +1342,7 @@
         <v>0</v>
       </c>
       <c r="Y7" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="Z7" t="n">
         <v>0</v>
@@ -1377,7 +1376,7 @@
       </c>
       <c r="AJ7" t="inlineStr">
         <is>
-          <t>sc34.png</t>
+          <t>sc32.png</t>
         </is>
       </c>
       <c r="AK7" t="inlineStr">
@@ -1393,7 +1392,7 @@
     </row>
     <row r="8">
       <c r="A8" t="n">
-        <v>22</v>
+        <v>15</v>
       </c>
       <c r="B8" t="inlineStr">
         <is>
@@ -1522,21 +1521,22 @@
     </row>
     <row r="9">
       <c r="A9" t="n">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>SC2-S27</t>
+          <t>SC2-S34</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Ego vehicle turns right at signalized junction</t>
+          <t>Ego vehicle turns right and ends up in same direction
+ as other vehicle at non-signalized junction</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>The ego vehicle is approaching a junction that is equipped with traffic light signals. The ego vehicle intends to turn right and other vehicle is going straight.</t>
+          <t xml:space="preserve">The ego vehicle is approaching a junction that is not equipped with traffic light signals. The ego vehicle intends to turn right at the junction. Another vehicle is approaching the junction from the left side of the ego vehicle. The other vehicle goes straight at the junction, such that it ends up in the same direction as the ego vehicle. </t>
         </is>
       </c>
       <c r="E9" t="n">
@@ -1579,7 +1579,7 @@
         <v>0</v>
       </c>
       <c r="R9" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="S9" t="n">
         <v>0</v>
@@ -1600,7 +1600,7 @@
         <v>0</v>
       </c>
       <c r="Y9" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="Z9" t="n">
         <v>0</v>
@@ -1624,17 +1624,17 @@
         <v>0</v>
       </c>
       <c r="AG9" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AH9" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AI9" t="n">
         <v>0</v>
       </c>
       <c r="AJ9" t="inlineStr">
         <is>
-          <t>sc261.png</t>
+          <t>sc34.png</t>
         </is>
       </c>
       <c r="AK9" t="inlineStr">
@@ -1650,21 +1650,22 @@
     </row>
     <row r="10">
       <c r="A10" t="n">
-        <v>19</v>
+        <v>17</v>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>SC2-S29</t>
+          <t>SC2-S35</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>Oncomingvehicle turns right at non-signalized junction</t>
+          <t xml:space="preserve"> Ego and crossing vehicle turn right at non-signalized
+ junction</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>The ego vehicle is approaching a junction that is not equipped with traffic light signals. It intended direction of the ego vehicle is not specified. Another vehicle is approaching the junction from the opposite direction. The other vehicle intends to turn right at the junction, such that the trajectories of the other vehicle and the ego vehicle might intersect</t>
+          <t>The ego vehicle is approaching a junction that is not equipped with traffic light signals. The ego vehicle intends to turn right at the junction. Another vehicle is approaching the junction from the left or right side of the ego vehicle. The other vehicle also turns right at the junction, such that the trajectories of the ego vehicle and the other vehicle intersect.</t>
         </is>
       </c>
       <c r="E10" t="n">
@@ -1762,7 +1763,7 @@
       </c>
       <c r="AJ10" t="inlineStr">
         <is>
-          <t>sc29.png</t>
+          <t>sc35.png</t>
         </is>
       </c>
       <c r="AK10" t="inlineStr">
@@ -1778,21 +1779,21 @@
     </row>
     <row r="11">
       <c r="A11" t="n">
-        <v>3</v>
+        <v>18</v>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>SC2-S9</t>
+          <t>SC2-S36</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Cut-in in front of the ego vehicle</t>
+          <t>Undertaking at left turn at non-signalized junction</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t xml:space="preserve">Another vehicle is driving in the same direction as the ego vehicle in an adjacent lane. The other vehicle makes a lane change, such that is becomes the lead vehicle from the ego vehicle’s perspective. </t>
+          <t xml:space="preserve">The ego vehicle is approaching a junction that is not equipped with traffic light signals. The ego vehicle intends to turn left at the junction. Another vehicle is driving in the same direction in the left lane next to the ego vehicle. </t>
         </is>
       </c>
       <c r="E11" t="n">
@@ -1883,14 +1884,14 @@
         <v>0</v>
       </c>
       <c r="AH11" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AI11" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AJ11" t="inlineStr">
         <is>
-          <t>sc9.png</t>
+          <t>sc36.png</t>
         </is>
       </c>
       <c r="AK11" t="inlineStr">
@@ -1900,27 +1901,28 @@
       </c>
       <c r="AL11" t="inlineStr">
         <is>
-          <t>Lane Change Scenario</t>
+          <t>Crossing Path</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="n">
-        <v>6</v>
+        <v>10</v>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>SC2-S12</t>
+          <t>SC2-S28</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>Cut-out in front of the ego vehicle</t>
+          <t>Ego vehicle turns right with oncoming vehicle at sig
+nalized junction</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>Another vehicle is driving in the same direction as the ego vehicle in front of the ego vehicle such that it is the lead vehicle from the ego vehicle’s perspective. The other vehicle makes a lane change, such that it will no longer be the ego vehicle’s lead vehicle.</t>
+          <t>The ego vehicle is approaching a junction that is equipped with traffic light signals. The ego vehicle turns right at the junction. Another vehicle is approaching the junction from the opposite direction. The other vehicle goes straight at the junction, such that the trajectories of the other vehicle and the ego vehicle intersect. The ego vehicle has to give right of way to the other vehicle.</t>
         </is>
       </c>
       <c r="E12" t="n">
@@ -1963,7 +1965,7 @@
         <v>0</v>
       </c>
       <c r="R12" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="S12" t="n">
         <v>0</v>
@@ -1984,7 +1986,7 @@
         <v>0</v>
       </c>
       <c r="Y12" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="Z12" t="n">
         <v>0</v>
@@ -2008,17 +2010,17 @@
         <v>0</v>
       </c>
       <c r="AG12" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AH12" t="n">
         <v>0</v>
       </c>
       <c r="AI12" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AJ12" t="inlineStr">
         <is>
-          <t>sc12.png</t>
+          <t>sc28.png</t>
         </is>
       </c>
       <c r="AK12" t="inlineStr">
@@ -2028,27 +2030,28 @@
       </c>
       <c r="AL12" t="inlineStr">
         <is>
-          <t>Lane Change Scenario</t>
+          <t>Opposite Direction</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="n">
-        <v>5</v>
+        <v>12</v>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>SC2-S11</t>
+          <t>SC2-S30</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>Ego merging into an occupied lane</t>
+          <t xml:space="preserve"> Ego vehicle turns right with oncoming vehicle at non
+signalized junction</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>The lane adjacent to the ego vehicle lane is occupied by slow driving vehicles. The ego vehicle intends to perform a lane change towards the lane in which the other vehicles are driving.</t>
+          <t xml:space="preserve">The ego vehicle is approaching a junction that is not equipped with traffic light signals. The ego vehicle intends to turn right at the junction. Another vehicle is approaching the junction from the opposite direction. The direction that the other vehicle goes to is not specified, i.e., the vehicle could turn left or right or the vehicle could go straight at the junction. </t>
         </is>
       </c>
       <c r="E13" t="n">
@@ -2103,7 +2106,7 @@
         <v>0</v>
       </c>
       <c r="V13" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="W13" t="n">
         <v>0</v>
@@ -2112,7 +2115,7 @@
         <v>0</v>
       </c>
       <c r="Y13" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="Z13" t="n">
         <v>0</v>
@@ -2139,14 +2142,14 @@
         <v>0</v>
       </c>
       <c r="AH13" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AI13" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AJ13" t="inlineStr">
         <is>
-          <t>sc11.png</t>
+          <t>sc30.png</t>
         </is>
       </c>
       <c r="AK13" t="inlineStr">
@@ -2156,27 +2159,28 @@
       </c>
       <c r="AL13" t="inlineStr">
         <is>
-          <t>Lane Change Scenario</t>
+          <t>Opposite Direction</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>SC2-S10</t>
+          <t>SC2-S1</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>Ego performing lane change with vehicle behind</t>
+          <t>Maneuvering a bend</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>Another vehicle is driving in the same direction as the ego vehicle, in a lane adjacent to the ego vehicle lane. The ego vehicle intends to perform a lane change towards the lane in which the other vehicle is driving</t>
+          <t>The ego vehicle is driving on a curved
+ road.</t>
         </is>
       </c>
       <c r="E14" t="n">
@@ -2222,7 +2226,7 @@
         <v>0</v>
       </c>
       <c r="S14" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="T14" t="n">
         <v>0</v>
@@ -2231,7 +2235,7 @@
         <v>0</v>
       </c>
       <c r="V14" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="W14" t="n">
         <v>0</v>
@@ -2274,7 +2278,7 @@
       </c>
       <c r="AJ14" t="inlineStr">
         <is>
-          <t>sc10.png</t>
+          <t>sc1.png</t>
         </is>
       </c>
       <c r="AK14" t="inlineStr">
@@ -2284,28 +2288,27 @@
       </c>
       <c r="AL14" t="inlineStr">
         <is>
-          <t>Lane Change Scenario</t>
+          <t>Turning Scenario</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="n">
-        <v>20</v>
+        <v>0</v>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>SC2-S30</t>
+          <t>SC2-S2</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t xml:space="preserve"> Ego vehicle turns right with oncoming vehicle at non
-signalized junction</t>
+          <t>Turning left</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t xml:space="preserve">The ego vehicle is approaching a junction that is not equipped with traffic light signals. The ego vehicle intends to turn right at the junction. Another vehicle is approaching the junction from the opposite direction. The direction that the other vehicle goes to is not specified, i.e., the vehicle could turn left or right or the vehicle could go straight at the junction. </t>
+          <t>The ego vehicle is turnning left at non-signalized junction.</t>
         </is>
       </c>
       <c r="E15" t="n">
@@ -2354,7 +2357,7 @@
         <v>0</v>
       </c>
       <c r="T15" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="U15" t="n">
         <v>0</v>
@@ -2369,7 +2372,7 @@
         <v>0</v>
       </c>
       <c r="Y15" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="Z15" t="n">
         <v>0</v>
@@ -2403,7 +2406,7 @@
       </c>
       <c r="AJ15" t="inlineStr">
         <is>
-          <t>sc30.png</t>
+          <t>sc2.png</t>
         </is>
       </c>
       <c r="AK15" t="inlineStr">
@@ -2413,27 +2416,27 @@
       </c>
       <c r="AL15" t="inlineStr">
         <is>
-          <t>Opposite Direction</t>
+          <t>Turning Scenario</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="n">
-        <v>12</v>
+        <v>1</v>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>SC2-S20</t>
+          <t>SC2-S3</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>Oncoming vehicle</t>
+          <t>Turning Right</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t xml:space="preserve">The ego vehicle is driving straight while another vehicle drives in opposite direction in the same lane. </t>
+          <t>The ego vehicle is turning right at non-signalized junction.</t>
         </is>
       </c>
       <c r="E16" t="n">
@@ -2476,7 +2479,7 @@
         <v>0</v>
       </c>
       <c r="R16" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="S16" t="n">
         <v>0</v>
@@ -2497,7 +2500,7 @@
         <v>0</v>
       </c>
       <c r="Y16" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="Z16" t="n">
         <v>0</v>
@@ -2524,14 +2527,14 @@
         <v>0</v>
       </c>
       <c r="AH16" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AI16" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AJ16" t="inlineStr">
         <is>
-          <t>sc20.png</t>
+          <t>sc3.png</t>
         </is>
       </c>
       <c r="AK16" t="inlineStr">
@@ -2541,28 +2544,27 @@
       </c>
       <c r="AL16" t="inlineStr">
         <is>
-          <t>Opposite Direction</t>
+          <t>Turning Scenario</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="n">
-        <v>18</v>
+        <v>2</v>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>SC2-S28</t>
+          <t>SC2-S5</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>Ego vehicle turns right with oncoming vehicle at sig
-nalized junction</t>
+          <t xml:space="preserve"> Navigating on an empty roundabout</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>The ego vehicle is approaching a junction that is equipped with traffic light signals. The ego vehicle turns right at the junction. Another vehicle is approaching the junction from the opposite direction. The other vehicle goes straight at the junction, such that the trajectories of the other vehicle and the ego vehicle intersect. The ego vehicle has to give right of way to the other vehicle.</t>
+          <t xml:space="preserve">The ego vehicle is approaching a round about. There are no other actors at the roundabout. The ego vehicle wants to navigate the roundabout in any of the possible directions. </t>
         </is>
       </c>
       <c r="E17" t="n">
@@ -2623,10 +2625,10 @@
         <v>0</v>
       </c>
       <c r="X17" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="Y17" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="Z17" t="n">
         <v>0</v>
@@ -2660,7 +2662,7 @@
       </c>
       <c r="AJ17" t="inlineStr">
         <is>
-          <t>sc28.png</t>
+          <t>sc5.png</t>
         </is>
       </c>
       <c r="AK17" t="inlineStr">
@@ -2670,40 +2672,34 @@
       </c>
       <c r="AL17" t="inlineStr">
         <is>
-          <t>Opposite Direction</t>
+          <t>Turning Scenario</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="n">
-        <v>33</v>
+        <v>4</v>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>SC2-S49</t>
+          <t>SC2-S16</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>Pedestrian at right turn at non-signalized junction</t>
+          <t>Vehicle backing up into ego vehicle</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>The ego vehicle is approaching a junction at which the ego vehicle intends to turn right. The junction is not equipped with traffic
-light signals. A pedestrian is walking on the right side of the ego vehicle. The walking
-direction of the pedestrian is not specified. Therefore, the pedestrian might walk towards
-the ego vehicle, in the same direction, or perpendicular to the ego vehicle, etc. Because the
-pedestrian is initially on the right side of the ego vehicle while the ego vehicle intends to
-turn right, it might be possible that the trajectories of the pedestrian and the ego vehicle
-intersect.</t>
+          <t>Another vehicle is driving in reverse. This could be, for example as shown in Figure 35a, because the vehicle is being parked. It might be the case that the ego vehicle has to respond to the reversing vehicle,</t>
         </is>
       </c>
       <c r="E18" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F18" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G18" t="n">
         <v>0</v>
@@ -2718,10 +2714,10 @@
         <v>0</v>
       </c>
       <c r="K18" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="L18" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="M18" t="n">
         <v>0</v>
@@ -2739,7 +2735,7 @@
         <v>0</v>
       </c>
       <c r="R18" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="S18" t="n">
         <v>0</v>
@@ -2760,7 +2756,7 @@
         <v>0</v>
       </c>
       <c r="Y18" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="Z18" t="n">
         <v>0</v>
@@ -2784,17 +2780,17 @@
         <v>0</v>
       </c>
       <c r="AG18" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AH18" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AI18" t="n">
         <v>0</v>
       </c>
       <c r="AJ18" t="inlineStr">
         <is>
-          <t>sc49.png</t>
+          <t>sc16.png</t>
         </is>
       </c>
       <c r="AK18" t="inlineStr">
@@ -2804,34 +2800,34 @@
       </c>
       <c r="AL18" t="inlineStr">
         <is>
-          <t>Pedestrian Interaction</t>
+          <t>Miscellaneous</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="n">
-        <v>27</v>
+        <v>5</v>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>SC2-S39</t>
+          <t>SC2-S23</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>Jaywalking</t>
+          <t xml:space="preserve"> Ego vehicle approaching red traffic light</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>The ego vehicle is driving on a road with a jaywalker. Although the jaywalker is not allowed to cross the road, the ego vehicle is expected to behave appropriately to avoid critical situations.</t>
+          <t>The ego vehicle is approaching a junction that is equipped with traffic light signals. The traffic signal for the ego vehicle is red. The objective of the ego vehicle is to cross the junction, but because the traffic signal is red, the ego vehicle is expected to stop.</t>
         </is>
       </c>
       <c r="E19" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F19" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G19" t="n">
         <v>0</v>
@@ -2912,17 +2908,17 @@
         <v>0</v>
       </c>
       <c r="AG19" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AH19" t="n">
         <v>0</v>
       </c>
       <c r="AI19" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AJ19" t="inlineStr">
         <is>
-          <t>sc39.png</t>
+          <t>sc23.png</t>
         </is>
       </c>
       <c r="AK19" t="inlineStr">
@@ -2932,34 +2928,34 @@
       </c>
       <c r="AL19" t="inlineStr">
         <is>
-          <t>Pedestrian Interaction</t>
+          <t>Traffic Signal</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="n">
-        <v>28</v>
+        <v>6</v>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>SC2-S40</t>
+          <t>SC2-S24</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>Pedestrian crossing at zebra crossing</t>
+          <t>Ego vehicle approaching green traffic light</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t xml:space="preserve">The ego vehicle is approaching a zebra crossing that is not equipped with traffic light signals. At the same time, a pedestrian is crossing the road using the zebra crossing. The ego vehicle has to give right of way to the pedestrian. </t>
+          <t>The ego vehicle is approaching a junction that is equipped with traffic light signals. The traffic signal for the ego vehicle is green or turns green. The objective of the ego vehicle is to cross the junction.</t>
         </is>
       </c>
       <c r="E20" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F20" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G20" t="n">
         <v>0</v>
@@ -3040,17 +3036,17 @@
         <v>0</v>
       </c>
       <c r="AG20" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AH20" t="n">
         <v>0</v>
       </c>
       <c r="AI20" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AJ20" t="inlineStr">
         <is>
-          <t>sc40.png</t>
+          <t>sc24.png</t>
         </is>
       </c>
       <c r="AK20" t="inlineStr">
@@ -3060,36 +3056,34 @@
       </c>
       <c r="AL20" t="inlineStr">
         <is>
-          <t>Pedestrian Interaction</t>
+          <t>Traffic Signal</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="n">
-        <v>29</v>
+        <v>7</v>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>SC2-S44</t>
+          <t>SC2-S25</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>Pedestrian running a red light</t>
+          <t xml:space="preserve"> Ego vehicle approaching amber traffic light</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>The ego vehicle is approaching a pedestrian crossing that is equipped with traffic light signals. The traffic signal for the ego vehicle
-is green. At the same time, a pedestrian is running through the red light. The ego vehicle
-might need to adopt its speed to stay at a safe distance from the pedestrian.</t>
+          <t>The ego vehicle is approaching a junction that is equipped with traffic light signals. The traffic signal for the ego vehicle is amber or turns amber. The objective of the ego vehicle is to cross the junction.</t>
         </is>
       </c>
       <c r="E21" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F21" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G21" t="n">
         <v>0</v>
@@ -3170,17 +3164,17 @@
         <v>0</v>
       </c>
       <c r="AG21" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AH21" t="n">
         <v>0</v>
       </c>
       <c r="AI21" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AJ21" t="inlineStr">
         <is>
-          <t>sc44.png</t>
+          <t>sc25.png</t>
         </is>
       </c>
       <c r="AK21" t="inlineStr">
@@ -3190,35 +3184,34 @@
       </c>
       <c r="AL21" t="inlineStr">
         <is>
-          <t>Pedestrian Interaction</t>
+          <t>Traffic Signal</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="n">
-        <v>30</v>
+        <v>8</v>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>SC2-S45</t>
+          <t>SC2-S26</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>Pedestrian crossing from behind an obstruction</t>
+          <t>Vehicle running red traffic light</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t xml:space="preserve">The ego vehicle is driving on a road while a pedestrian crosses the road. The pedestrian is initially outside the view of the ego
-vehicle due to an obstruction. </t>
+          <t xml:space="preserve">The ego vehicle is approaching a junction that is equipped with traffic light signals. The traffic signal for the ego vehicle is green. Another vehicle is also approaching the junction and its trajectory intersects that of the ego vehicle. The traffic signal for the other vehicle is red. However, the vehicle is running through the red light. </t>
         </is>
       </c>
       <c r="E22" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F22" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G22" t="n">
         <v>0</v>
@@ -3299,17 +3292,17 @@
         <v>0</v>
       </c>
       <c r="AG22" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AH22" t="n">
         <v>0</v>
       </c>
       <c r="AI22" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AJ22" t="inlineStr">
         <is>
-          <t>sc45.png</t>
+          <t>sc26.png</t>
         </is>
       </c>
       <c r="AK22" t="inlineStr">
@@ -3319,36 +3312,34 @@
       </c>
       <c r="AL22" t="inlineStr">
         <is>
-          <t>Pedestrian Interaction</t>
+          <t>Traffic Signal</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="n">
-        <v>31</v>
+        <v>19</v>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>SC2-S46</t>
+          <t>SC2-S37</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>Pedestrian at left turn at non-signalized junction</t>
+          <t>Entering a roundabout with another vehicle</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t xml:space="preserve">The ego vehicle is approaching a junction at which the ego vehicle intends to turn left. The junction is not equipped with traffic light
-signals. A pedestrian is walking on the left side of the ego vehicle. The walking direction of
-the pedestrian is not specified. </t>
+          <t>The ego vehicle is approaching a round about. There is another vehicle on the roundabout or another vehicle is approaching the roundabout from another direction.</t>
         </is>
       </c>
       <c r="E23" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F23" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G23" t="n">
         <v>0</v>
@@ -3384,13 +3375,13 @@
         <v>0</v>
       </c>
       <c r="R23" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="S23" t="n">
         <v>0</v>
       </c>
       <c r="T23" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="U23" t="n">
         <v>0</v>
@@ -3439,7 +3430,7 @@
       </c>
       <c r="AJ23" t="inlineStr">
         <is>
-          <t>sc46.png</t>
+          <t>sc37.png</t>
         </is>
       </c>
       <c r="AK23" t="inlineStr">
@@ -3448,1809 +3439,6 @@
         </is>
       </c>
       <c r="AL23" t="inlineStr">
-        <is>
-          <t>Pedestrian Interaction</t>
-        </is>
-      </c>
-    </row>
-    <row r="24">
-      <c r="A24" t="n">
-        <v>32</v>
-      </c>
-      <c r="B24" t="inlineStr">
-        <is>
-          <t>SC2-S48</t>
-        </is>
-      </c>
-      <c r="C24" t="inlineStr">
-        <is>
-          <t>Pedestrian in same direction obstructed at ego left turn</t>
-        </is>
-      </c>
-      <c r="D24" t="inlineStr">
-        <is>
-          <t>The ego vehicle is approaching a junction at which the ego vehicle intends to turn left. It is not specified whether the junction is
-equipped with traffic light signals. A pedestrian is approaching the junction from the same
-direction on the left side of the road (from the perspective of the ego vehicle). The pedestrian
-goes straight at the junction such that the trajectories of the ego vehicle and the pedestrian
-intersect. The view from the ego vehicle to the pedestrian is obstructed, e.g., by bushes or
-a hedge.</t>
-        </is>
-      </c>
-      <c r="E24" t="n">
-        <v>0</v>
-      </c>
-      <c r="F24" t="n">
-        <v>1</v>
-      </c>
-      <c r="G24" t="n">
-        <v>0</v>
-      </c>
-      <c r="H24" t="n">
-        <v>0</v>
-      </c>
-      <c r="I24" t="n">
-        <v>0</v>
-      </c>
-      <c r="J24" t="n">
-        <v>0</v>
-      </c>
-      <c r="K24" t="n">
-        <v>1</v>
-      </c>
-      <c r="L24" t="n">
-        <v>0</v>
-      </c>
-      <c r="M24" t="n">
-        <v>0</v>
-      </c>
-      <c r="N24" t="n">
-        <v>0</v>
-      </c>
-      <c r="O24" t="n">
-        <v>1</v>
-      </c>
-      <c r="P24" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q24" t="n">
-        <v>0</v>
-      </c>
-      <c r="R24" t="n">
-        <v>0</v>
-      </c>
-      <c r="S24" t="n">
-        <v>0</v>
-      </c>
-      <c r="T24" t="n">
-        <v>1</v>
-      </c>
-      <c r="U24" t="n">
-        <v>0</v>
-      </c>
-      <c r="V24" t="n">
-        <v>0</v>
-      </c>
-      <c r="W24" t="n">
-        <v>0</v>
-      </c>
-      <c r="X24" t="n">
-        <v>0</v>
-      </c>
-      <c r="Y24" t="n">
-        <v>0</v>
-      </c>
-      <c r="Z24" t="n">
-        <v>0</v>
-      </c>
-      <c r="AA24" t="n">
-        <v>0</v>
-      </c>
-      <c r="AB24" t="n">
-        <v>0</v>
-      </c>
-      <c r="AC24" t="n">
-        <v>0</v>
-      </c>
-      <c r="AD24" t="n">
-        <v>0</v>
-      </c>
-      <c r="AE24" t="n">
-        <v>0</v>
-      </c>
-      <c r="AF24" t="n">
-        <v>0</v>
-      </c>
-      <c r="AG24" t="n">
-        <v>0</v>
-      </c>
-      <c r="AH24" t="n">
-        <v>1</v>
-      </c>
-      <c r="AI24" t="n">
-        <v>0</v>
-      </c>
-      <c r="AJ24" t="inlineStr">
-        <is>
-          <t>sc48.png</t>
-        </is>
-      </c>
-      <c r="AK24" t="inlineStr">
-        <is>
-          <t>Singapore</t>
-        </is>
-      </c>
-      <c r="AL24" t="inlineStr">
-        <is>
-          <t>Pedestrian Interaction</t>
-        </is>
-      </c>
-    </row>
-    <row r="25">
-      <c r="A25" t="n">
-        <v>34</v>
-      </c>
-      <c r="B25" t="inlineStr">
-        <is>
-          <t>SC2-S50</t>
-        </is>
-      </c>
-      <c r="C25" t="inlineStr">
-        <is>
-          <t>Pedestrian at right turn at signalized junction</t>
-        </is>
-      </c>
-      <c r="D25" t="inlineStr">
-        <is>
-          <t>The ego vehicle is approaching a junction at which the ego vehicle intends to turn right. The junction is equipped with traffic light
-signals. A pedestrian is walking on the right side of the ego vehicle. The walking direction of
-the pedestrian is not specified. Therefore, the pedestrian might walk towards the ego vehicle,
-in the same direction, or perpendicular to the ego vehicle, etc. Because the pedestrian is
-initially on the right side of the ego vehicle while the ego vehicle intends to turn right, it
-might be possible that the trajectories of the pedestrian and the ego vehicle intersect</t>
-        </is>
-      </c>
-      <c r="E25" t="n">
-        <v>0</v>
-      </c>
-      <c r="F25" t="n">
-        <v>1</v>
-      </c>
-      <c r="G25" t="n">
-        <v>0</v>
-      </c>
-      <c r="H25" t="n">
-        <v>0</v>
-      </c>
-      <c r="I25" t="n">
-        <v>0</v>
-      </c>
-      <c r="J25" t="n">
-        <v>0</v>
-      </c>
-      <c r="K25" t="n">
-        <v>1</v>
-      </c>
-      <c r="L25" t="n">
-        <v>0</v>
-      </c>
-      <c r="M25" t="n">
-        <v>0</v>
-      </c>
-      <c r="N25" t="n">
-        <v>0</v>
-      </c>
-      <c r="O25" t="n">
-        <v>1</v>
-      </c>
-      <c r="P25" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q25" t="n">
-        <v>0</v>
-      </c>
-      <c r="R25" t="n">
-        <v>0</v>
-      </c>
-      <c r="S25" t="n">
-        <v>0</v>
-      </c>
-      <c r="T25" t="n">
-        <v>0</v>
-      </c>
-      <c r="U25" t="n">
-        <v>0</v>
-      </c>
-      <c r="V25" t="n">
-        <v>0</v>
-      </c>
-      <c r="W25" t="n">
-        <v>0</v>
-      </c>
-      <c r="X25" t="n">
-        <v>0</v>
-      </c>
-      <c r="Y25" t="n">
-        <v>1</v>
-      </c>
-      <c r="Z25" t="n">
-        <v>0</v>
-      </c>
-      <c r="AA25" t="n">
-        <v>0</v>
-      </c>
-      <c r="AB25" t="n">
-        <v>0</v>
-      </c>
-      <c r="AC25" t="n">
-        <v>0</v>
-      </c>
-      <c r="AD25" t="n">
-        <v>0</v>
-      </c>
-      <c r="AE25" t="n">
-        <v>0</v>
-      </c>
-      <c r="AF25" t="n">
-        <v>0</v>
-      </c>
-      <c r="AG25" t="n">
-        <v>1</v>
-      </c>
-      <c r="AH25" t="n">
-        <v>0</v>
-      </c>
-      <c r="AI25" t="n">
-        <v>0</v>
-      </c>
-      <c r="AJ25" t="inlineStr">
-        <is>
-          <t>sc50.png</t>
-        </is>
-      </c>
-      <c r="AK25" t="inlineStr">
-        <is>
-          <t>Singapore</t>
-        </is>
-      </c>
-      <c r="AL25" t="inlineStr">
-        <is>
-          <t>Pedestrian Interaction</t>
-        </is>
-      </c>
-    </row>
-    <row r="26">
-      <c r="A26" t="n">
-        <v>1</v>
-      </c>
-      <c r="B26" t="inlineStr">
-        <is>
-          <t>SC2-S1</t>
-        </is>
-      </c>
-      <c r="C26" t="inlineStr">
-        <is>
-          <t>Maneuvering a bend</t>
-        </is>
-      </c>
-      <c r="D26" t="inlineStr">
-        <is>
-          <t>The ego vehicle is driving on a curved
- road.</t>
-        </is>
-      </c>
-      <c r="E26" t="n">
-        <v>1</v>
-      </c>
-      <c r="F26" t="n">
-        <v>0</v>
-      </c>
-      <c r="G26" t="n">
-        <v>0</v>
-      </c>
-      <c r="H26" t="n">
-        <v>0</v>
-      </c>
-      <c r="I26" t="n">
-        <v>0</v>
-      </c>
-      <c r="J26" t="n">
-        <v>0</v>
-      </c>
-      <c r="K26" t="n">
-        <v>1</v>
-      </c>
-      <c r="L26" t="n">
-        <v>0</v>
-      </c>
-      <c r="M26" t="n">
-        <v>0</v>
-      </c>
-      <c r="N26" t="n">
-        <v>0</v>
-      </c>
-      <c r="O26" t="n">
-        <v>1</v>
-      </c>
-      <c r="P26" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q26" t="n">
-        <v>0</v>
-      </c>
-      <c r="R26" t="n">
-        <v>0</v>
-      </c>
-      <c r="S26" t="n">
-        <v>1</v>
-      </c>
-      <c r="T26" t="n">
-        <v>0</v>
-      </c>
-      <c r="U26" t="n">
-        <v>0</v>
-      </c>
-      <c r="V26" t="n">
-        <v>0</v>
-      </c>
-      <c r="W26" t="n">
-        <v>0</v>
-      </c>
-      <c r="X26" t="n">
-        <v>0</v>
-      </c>
-      <c r="Y26" t="n">
-        <v>0</v>
-      </c>
-      <c r="Z26" t="n">
-        <v>0</v>
-      </c>
-      <c r="AA26" t="n">
-        <v>0</v>
-      </c>
-      <c r="AB26" t="n">
-        <v>0</v>
-      </c>
-      <c r="AC26" t="n">
-        <v>0</v>
-      </c>
-      <c r="AD26" t="n">
-        <v>0</v>
-      </c>
-      <c r="AE26" t="n">
-        <v>0</v>
-      </c>
-      <c r="AF26" t="n">
-        <v>0</v>
-      </c>
-      <c r="AG26" t="n">
-        <v>0</v>
-      </c>
-      <c r="AH26" t="n">
-        <v>0</v>
-      </c>
-      <c r="AI26" t="n">
-        <v>1</v>
-      </c>
-      <c r="AJ26" t="inlineStr">
-        <is>
-          <t>sc1.png</t>
-        </is>
-      </c>
-      <c r="AK26" t="inlineStr">
-        <is>
-          <t>Singapore</t>
-        </is>
-      </c>
-      <c r="AL26" t="inlineStr">
-        <is>
-          <t>Turning Scenario</t>
-        </is>
-      </c>
-    </row>
-    <row r="27">
-      <c r="A27" t="n">
-        <v>0</v>
-      </c>
-      <c r="B27" t="inlineStr">
-        <is>
-          <t>SC2-S2</t>
-        </is>
-      </c>
-      <c r="C27" t="inlineStr">
-        <is>
-          <t>Turning left</t>
-        </is>
-      </c>
-      <c r="D27" t="inlineStr">
-        <is>
-          <t>The ego vehicle is turnning left at non-signalized junction.</t>
-        </is>
-      </c>
-      <c r="E27" t="n">
-        <v>1</v>
-      </c>
-      <c r="F27" t="n">
-        <v>0</v>
-      </c>
-      <c r="G27" t="n">
-        <v>0</v>
-      </c>
-      <c r="H27" t="n">
-        <v>0</v>
-      </c>
-      <c r="I27" t="n">
-        <v>0</v>
-      </c>
-      <c r="J27" t="n">
-        <v>0</v>
-      </c>
-      <c r="K27" t="n">
-        <v>1</v>
-      </c>
-      <c r="L27" t="n">
-        <v>0</v>
-      </c>
-      <c r="M27" t="n">
-        <v>0</v>
-      </c>
-      <c r="N27" t="n">
-        <v>0</v>
-      </c>
-      <c r="O27" t="n">
-        <v>1</v>
-      </c>
-      <c r="P27" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q27" t="n">
-        <v>0</v>
-      </c>
-      <c r="R27" t="n">
-        <v>0</v>
-      </c>
-      <c r="S27" t="n">
-        <v>0</v>
-      </c>
-      <c r="T27" t="n">
-        <v>1</v>
-      </c>
-      <c r="U27" t="n">
-        <v>0</v>
-      </c>
-      <c r="V27" t="n">
-        <v>0</v>
-      </c>
-      <c r="W27" t="n">
-        <v>0</v>
-      </c>
-      <c r="X27" t="n">
-        <v>0</v>
-      </c>
-      <c r="Y27" t="n">
-        <v>0</v>
-      </c>
-      <c r="Z27" t="n">
-        <v>0</v>
-      </c>
-      <c r="AA27" t="n">
-        <v>0</v>
-      </c>
-      <c r="AB27" t="n">
-        <v>0</v>
-      </c>
-      <c r="AC27" t="n">
-        <v>0</v>
-      </c>
-      <c r="AD27" t="n">
-        <v>0</v>
-      </c>
-      <c r="AE27" t="n">
-        <v>0</v>
-      </c>
-      <c r="AF27" t="n">
-        <v>0</v>
-      </c>
-      <c r="AG27" t="n">
-        <v>0</v>
-      </c>
-      <c r="AH27" t="n">
-        <v>1</v>
-      </c>
-      <c r="AI27" t="n">
-        <v>0</v>
-      </c>
-      <c r="AJ27" t="inlineStr">
-        <is>
-          <t>sc2.png</t>
-        </is>
-      </c>
-      <c r="AK27" t="inlineStr">
-        <is>
-          <t>Singapore</t>
-        </is>
-      </c>
-      <c r="AL27" t="inlineStr">
-        <is>
-          <t>Turning Scenario</t>
-        </is>
-      </c>
-    </row>
-    <row r="28">
-      <c r="A28" t="n">
-        <v>1</v>
-      </c>
-      <c r="B28" t="inlineStr">
-        <is>
-          <t>SC2-S3</t>
-        </is>
-      </c>
-      <c r="C28" t="inlineStr">
-        <is>
-          <t>Turning Right</t>
-        </is>
-      </c>
-      <c r="D28" t="inlineStr">
-        <is>
-          <t>The ego vehicle is turning right at non-signalized junction.</t>
-        </is>
-      </c>
-      <c r="E28" t="n">
-        <v>1</v>
-      </c>
-      <c r="F28" t="n">
-        <v>0</v>
-      </c>
-      <c r="G28" t="n">
-        <v>0</v>
-      </c>
-      <c r="H28" t="n">
-        <v>0</v>
-      </c>
-      <c r="I28" t="n">
-        <v>0</v>
-      </c>
-      <c r="J28" t="n">
-        <v>0</v>
-      </c>
-      <c r="K28" t="n">
-        <v>1</v>
-      </c>
-      <c r="L28" t="n">
-        <v>0</v>
-      </c>
-      <c r="M28" t="n">
-        <v>0</v>
-      </c>
-      <c r="N28" t="n">
-        <v>0</v>
-      </c>
-      <c r="O28" t="n">
-        <v>1</v>
-      </c>
-      <c r="P28" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q28" t="n">
-        <v>0</v>
-      </c>
-      <c r="R28" t="n">
-        <v>0</v>
-      </c>
-      <c r="S28" t="n">
-        <v>0</v>
-      </c>
-      <c r="T28" t="n">
-        <v>0</v>
-      </c>
-      <c r="U28" t="n">
-        <v>0</v>
-      </c>
-      <c r="V28" t="n">
-        <v>0</v>
-      </c>
-      <c r="W28" t="n">
-        <v>0</v>
-      </c>
-      <c r="X28" t="n">
-        <v>0</v>
-      </c>
-      <c r="Y28" t="n">
-        <v>1</v>
-      </c>
-      <c r="Z28" t="n">
-        <v>0</v>
-      </c>
-      <c r="AA28" t="n">
-        <v>0</v>
-      </c>
-      <c r="AB28" t="n">
-        <v>0</v>
-      </c>
-      <c r="AC28" t="n">
-        <v>0</v>
-      </c>
-      <c r="AD28" t="n">
-        <v>0</v>
-      </c>
-      <c r="AE28" t="n">
-        <v>0</v>
-      </c>
-      <c r="AF28" t="n">
-        <v>0</v>
-      </c>
-      <c r="AG28" t="n">
-        <v>0</v>
-      </c>
-      <c r="AH28" t="n">
-        <v>1</v>
-      </c>
-      <c r="AI28" t="n">
-        <v>0</v>
-      </c>
-      <c r="AJ28" t="inlineStr">
-        <is>
-          <t>sc3.png</t>
-        </is>
-      </c>
-      <c r="AK28" t="inlineStr">
-        <is>
-          <t>Singapore</t>
-        </is>
-      </c>
-      <c r="AL28" t="inlineStr">
-        <is>
-          <t>Turning Scenario</t>
-        </is>
-      </c>
-    </row>
-    <row r="29">
-      <c r="A29" t="n">
-        <v>2</v>
-      </c>
-      <c r="B29" t="inlineStr">
-        <is>
-          <t>SC2-S5</t>
-        </is>
-      </c>
-      <c r="C29" t="inlineStr">
-        <is>
-          <t xml:space="preserve"> Navigating on an empty roundabout</t>
-        </is>
-      </c>
-      <c r="D29" t="inlineStr">
-        <is>
-          <t xml:space="preserve">The ego vehicle is approaching a round about. There are no other actors at the roundabout. The ego vehicle wants to navigate the roundabout in any of the possible directions. </t>
-        </is>
-      </c>
-      <c r="E29" t="n">
-        <v>1</v>
-      </c>
-      <c r="F29" t="n">
-        <v>0</v>
-      </c>
-      <c r="G29" t="n">
-        <v>0</v>
-      </c>
-      <c r="H29" t="n">
-        <v>0</v>
-      </c>
-      <c r="I29" t="n">
-        <v>0</v>
-      </c>
-      <c r="J29" t="n">
-        <v>0</v>
-      </c>
-      <c r="K29" t="n">
-        <v>1</v>
-      </c>
-      <c r="L29" t="n">
-        <v>0</v>
-      </c>
-      <c r="M29" t="n">
-        <v>0</v>
-      </c>
-      <c r="N29" t="n">
-        <v>0</v>
-      </c>
-      <c r="O29" t="n">
-        <v>1</v>
-      </c>
-      <c r="P29" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q29" t="n">
-        <v>0</v>
-      </c>
-      <c r="R29" t="n">
-        <v>0</v>
-      </c>
-      <c r="S29" t="n">
-        <v>0</v>
-      </c>
-      <c r="T29" t="n">
-        <v>0</v>
-      </c>
-      <c r="U29" t="n">
-        <v>0</v>
-      </c>
-      <c r="V29" t="n">
-        <v>0</v>
-      </c>
-      <c r="W29" t="n">
-        <v>0</v>
-      </c>
-      <c r="X29" t="n">
-        <v>1</v>
-      </c>
-      <c r="Y29" t="n">
-        <v>0</v>
-      </c>
-      <c r="Z29" t="n">
-        <v>0</v>
-      </c>
-      <c r="AA29" t="n">
-        <v>0</v>
-      </c>
-      <c r="AB29" t="n">
-        <v>0</v>
-      </c>
-      <c r="AC29" t="n">
-        <v>0</v>
-      </c>
-      <c r="AD29" t="n">
-        <v>0</v>
-      </c>
-      <c r="AE29" t="n">
-        <v>0</v>
-      </c>
-      <c r="AF29" t="n">
-        <v>0</v>
-      </c>
-      <c r="AG29" t="n">
-        <v>1</v>
-      </c>
-      <c r="AH29" t="n">
-        <v>0</v>
-      </c>
-      <c r="AI29" t="n">
-        <v>0</v>
-      </c>
-      <c r="AJ29" t="inlineStr">
-        <is>
-          <t>sc5.png</t>
-        </is>
-      </c>
-      <c r="AK29" t="inlineStr">
-        <is>
-          <t>Singapore</t>
-        </is>
-      </c>
-      <c r="AL29" t="inlineStr">
-        <is>
-          <t>Turning Scenario</t>
-        </is>
-      </c>
-    </row>
-    <row r="30">
-      <c r="A30" t="n">
-        <v>9</v>
-      </c>
-      <c r="B30" t="inlineStr">
-        <is>
-          <t>SC2-S17</t>
-        </is>
-      </c>
-      <c r="C30" t="inlineStr">
-        <is>
-          <t>Stopping at a bus bay</t>
-        </is>
-      </c>
-      <c r="D30" t="inlineStr">
-        <is>
-          <t xml:space="preserve">The ego vehicle is approaching a bus bay. The goal of the ego vehicle is to park at the bus bay. </t>
-        </is>
-      </c>
-      <c r="E30" t="n">
-        <v>1</v>
-      </c>
-      <c r="F30" t="n">
-        <v>0</v>
-      </c>
-      <c r="G30" t="n">
-        <v>0</v>
-      </c>
-      <c r="H30" t="n">
-        <v>0</v>
-      </c>
-      <c r="I30" t="n">
-        <v>0</v>
-      </c>
-      <c r="J30" t="n">
-        <v>0</v>
-      </c>
-      <c r="K30" t="n">
-        <v>1</v>
-      </c>
-      <c r="L30" t="n">
-        <v>0</v>
-      </c>
-      <c r="M30" t="n">
-        <v>0</v>
-      </c>
-      <c r="N30" t="n">
-        <v>0</v>
-      </c>
-      <c r="O30" t="n">
-        <v>1</v>
-      </c>
-      <c r="P30" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q30" t="n">
-        <v>0</v>
-      </c>
-      <c r="R30" t="n">
-        <v>1</v>
-      </c>
-      <c r="S30" t="n">
-        <v>0</v>
-      </c>
-      <c r="T30" t="n">
-        <v>0</v>
-      </c>
-      <c r="U30" t="n">
-        <v>0</v>
-      </c>
-      <c r="V30" t="n">
-        <v>0</v>
-      </c>
-      <c r="W30" t="n">
-        <v>0</v>
-      </c>
-      <c r="X30" t="n">
-        <v>0</v>
-      </c>
-      <c r="Y30" t="n">
-        <v>0</v>
-      </c>
-      <c r="Z30" t="n">
-        <v>0</v>
-      </c>
-      <c r="AA30" t="n">
-        <v>0</v>
-      </c>
-      <c r="AB30" t="n">
-        <v>0</v>
-      </c>
-      <c r="AC30" t="n">
-        <v>0</v>
-      </c>
-      <c r="AD30" t="n">
-        <v>0</v>
-      </c>
-      <c r="AE30" t="n">
-        <v>0</v>
-      </c>
-      <c r="AF30" t="n">
-        <v>0</v>
-      </c>
-      <c r="AG30" t="n">
-        <v>0</v>
-      </c>
-      <c r="AH30" t="n">
-        <v>0</v>
-      </c>
-      <c r="AI30" t="n">
-        <v>1</v>
-      </c>
-      <c r="AJ30" t="inlineStr">
-        <is>
-          <t>sc17.png</t>
-        </is>
-      </c>
-      <c r="AK30" t="inlineStr">
-        <is>
-          <t>Singapore</t>
-        </is>
-      </c>
-      <c r="AL30" t="inlineStr">
-        <is>
-          <t>Miscellaneous</t>
-        </is>
-      </c>
-    </row>
-    <row r="31">
-      <c r="A31" t="n">
-        <v>10</v>
-      </c>
-      <c r="B31" t="inlineStr">
-        <is>
-          <t>SC2-S18</t>
-        </is>
-      </c>
-      <c r="C31" t="inlineStr">
-        <is>
-          <t>Leaving a bus bay</t>
-        </is>
-      </c>
-      <c r="D31" t="inlineStr">
-        <is>
-          <t>The ego vehicle is initially stationary at a bus bay. The goal of the ego vehicle is to leave the bus bay.</t>
-        </is>
-      </c>
-      <c r="E31" t="n">
-        <v>1</v>
-      </c>
-      <c r="F31" t="n">
-        <v>0</v>
-      </c>
-      <c r="G31" t="n">
-        <v>0</v>
-      </c>
-      <c r="H31" t="n">
-        <v>0</v>
-      </c>
-      <c r="I31" t="n">
-        <v>0</v>
-      </c>
-      <c r="J31" t="n">
-        <v>0</v>
-      </c>
-      <c r="K31" t="n">
-        <v>1</v>
-      </c>
-      <c r="L31" t="n">
-        <v>0</v>
-      </c>
-      <c r="M31" t="n">
-        <v>0</v>
-      </c>
-      <c r="N31" t="n">
-        <v>0</v>
-      </c>
-      <c r="O31" t="n">
-        <v>1</v>
-      </c>
-      <c r="P31" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q31" t="n">
-        <v>0</v>
-      </c>
-      <c r="R31" t="n">
-        <v>0</v>
-      </c>
-      <c r="S31" t="n">
-        <v>0</v>
-      </c>
-      <c r="T31" t="n">
-        <v>0</v>
-      </c>
-      <c r="U31" t="n">
-        <v>0</v>
-      </c>
-      <c r="V31" t="n">
-        <v>0</v>
-      </c>
-      <c r="W31" t="n">
-        <v>1</v>
-      </c>
-      <c r="X31" t="n">
-        <v>0</v>
-      </c>
-      <c r="Y31" t="n">
-        <v>0</v>
-      </c>
-      <c r="Z31" t="n">
-        <v>0</v>
-      </c>
-      <c r="AA31" t="n">
-        <v>0</v>
-      </c>
-      <c r="AB31" t="n">
-        <v>0</v>
-      </c>
-      <c r="AC31" t="n">
-        <v>0</v>
-      </c>
-      <c r="AD31" t="n">
-        <v>0</v>
-      </c>
-      <c r="AE31" t="n">
-        <v>0</v>
-      </c>
-      <c r="AF31" t="n">
-        <v>0</v>
-      </c>
-      <c r="AG31" t="n">
-        <v>0</v>
-      </c>
-      <c r="AH31" t="n">
-        <v>0</v>
-      </c>
-      <c r="AI31" t="n">
-        <v>1</v>
-      </c>
-      <c r="AJ31" t="inlineStr">
-        <is>
-          <t>sc18.png</t>
-        </is>
-      </c>
-      <c r="AK31" t="inlineStr">
-        <is>
-          <t>Singapore</t>
-        </is>
-      </c>
-      <c r="AL31" t="inlineStr">
-        <is>
-          <t>Miscellaneous</t>
-        </is>
-      </c>
-    </row>
-    <row r="32">
-      <c r="A32" t="n">
-        <v>11</v>
-      </c>
-      <c r="B32" t="inlineStr">
-        <is>
-          <t>SC2-S19</t>
-        </is>
-      </c>
-      <c r="C32" t="inlineStr">
-        <is>
-          <t xml:space="preserve"> Driving along a bus bay</t>
-        </is>
-      </c>
-      <c r="D32" t="inlineStr">
-        <is>
-          <t>The ego vehicle passes a bus bay. The goal of the ego vehicle is to continue driving. There might be another vehicle at the bus bay intending to leave the bus bay.</t>
-        </is>
-      </c>
-      <c r="E32" t="n">
-        <v>1</v>
-      </c>
-      <c r="F32" t="n">
-        <v>0</v>
-      </c>
-      <c r="G32" t="n">
-        <v>0</v>
-      </c>
-      <c r="H32" t="n">
-        <v>0</v>
-      </c>
-      <c r="I32" t="n">
-        <v>0</v>
-      </c>
-      <c r="J32" t="n">
-        <v>0</v>
-      </c>
-      <c r="K32" t="n">
-        <v>1</v>
-      </c>
-      <c r="L32" t="n">
-        <v>0</v>
-      </c>
-      <c r="M32" t="n">
-        <v>0</v>
-      </c>
-      <c r="N32" t="n">
-        <v>0</v>
-      </c>
-      <c r="O32" t="n">
-        <v>1</v>
-      </c>
-      <c r="P32" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q32" t="n">
-        <v>0</v>
-      </c>
-      <c r="R32" t="n">
-        <v>1</v>
-      </c>
-      <c r="S32" t="n">
-        <v>0</v>
-      </c>
-      <c r="T32" t="n">
-        <v>0</v>
-      </c>
-      <c r="U32" t="n">
-        <v>0</v>
-      </c>
-      <c r="V32" t="n">
-        <v>0</v>
-      </c>
-      <c r="W32" t="n">
-        <v>0</v>
-      </c>
-      <c r="X32" t="n">
-        <v>0</v>
-      </c>
-      <c r="Y32" t="n">
-        <v>0</v>
-      </c>
-      <c r="Z32" t="n">
-        <v>0</v>
-      </c>
-      <c r="AA32" t="n">
-        <v>0</v>
-      </c>
-      <c r="AB32" t="n">
-        <v>0</v>
-      </c>
-      <c r="AC32" t="n">
-        <v>0</v>
-      </c>
-      <c r="AD32" t="n">
-        <v>0</v>
-      </c>
-      <c r="AE32" t="n">
-        <v>0</v>
-      </c>
-      <c r="AF32" t="n">
-        <v>0</v>
-      </c>
-      <c r="AG32" t="n">
-        <v>0</v>
-      </c>
-      <c r="AH32" t="n">
-        <v>0</v>
-      </c>
-      <c r="AI32" t="n">
-        <v>1</v>
-      </c>
-      <c r="AJ32" t="inlineStr">
-        <is>
-          <t>sc19.png</t>
-        </is>
-      </c>
-      <c r="AK32" t="inlineStr">
-        <is>
-          <t>Singapore</t>
-        </is>
-      </c>
-      <c r="AL32" t="inlineStr">
-        <is>
-          <t>Miscellaneous</t>
-        </is>
-      </c>
-    </row>
-    <row r="33">
-      <c r="A33" t="n">
-        <v>13</v>
-      </c>
-      <c r="B33" t="inlineStr">
-        <is>
-          <t>SC2-S23</t>
-        </is>
-      </c>
-      <c r="C33" t="inlineStr">
-        <is>
-          <t xml:space="preserve"> Ego vehicle approaching red traffic light</t>
-        </is>
-      </c>
-      <c r="D33" t="inlineStr">
-        <is>
-          <t>The ego vehicle is approaching a junction that is equipped with traffic light signals. The traffic signal for the ego vehicle is red. The objective of the ego vehicle is to cross the junction, but because the traffic signal is red, the ego vehicle is expected to stop.</t>
-        </is>
-      </c>
-      <c r="E33" t="n">
-        <v>1</v>
-      </c>
-      <c r="F33" t="n">
-        <v>0</v>
-      </c>
-      <c r="G33" t="n">
-        <v>0</v>
-      </c>
-      <c r="H33" t="n">
-        <v>0</v>
-      </c>
-      <c r="I33" t="n">
-        <v>0</v>
-      </c>
-      <c r="J33" t="n">
-        <v>0</v>
-      </c>
-      <c r="K33" t="n">
-        <v>1</v>
-      </c>
-      <c r="L33" t="n">
-        <v>0</v>
-      </c>
-      <c r="M33" t="n">
-        <v>0</v>
-      </c>
-      <c r="N33" t="n">
-        <v>0</v>
-      </c>
-      <c r="O33" t="n">
-        <v>1</v>
-      </c>
-      <c r="P33" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q33" t="n">
-        <v>0</v>
-      </c>
-      <c r="R33" t="n">
-        <v>1</v>
-      </c>
-      <c r="S33" t="n">
-        <v>0</v>
-      </c>
-      <c r="T33" t="n">
-        <v>0</v>
-      </c>
-      <c r="U33" t="n">
-        <v>0</v>
-      </c>
-      <c r="V33" t="n">
-        <v>0</v>
-      </c>
-      <c r="W33" t="n">
-        <v>0</v>
-      </c>
-      <c r="X33" t="n">
-        <v>0</v>
-      </c>
-      <c r="Y33" t="n">
-        <v>0</v>
-      </c>
-      <c r="Z33" t="n">
-        <v>0</v>
-      </c>
-      <c r="AA33" t="n">
-        <v>0</v>
-      </c>
-      <c r="AB33" t="n">
-        <v>0</v>
-      </c>
-      <c r="AC33" t="n">
-        <v>0</v>
-      </c>
-      <c r="AD33" t="n">
-        <v>0</v>
-      </c>
-      <c r="AE33" t="n">
-        <v>0</v>
-      </c>
-      <c r="AF33" t="n">
-        <v>0</v>
-      </c>
-      <c r="AG33" t="n">
-        <v>1</v>
-      </c>
-      <c r="AH33" t="n">
-        <v>0</v>
-      </c>
-      <c r="AI33" t="n">
-        <v>0</v>
-      </c>
-      <c r="AJ33" t="inlineStr">
-        <is>
-          <t>sc23.png</t>
-        </is>
-      </c>
-      <c r="AK33" t="inlineStr">
-        <is>
-          <t>Singapore</t>
-        </is>
-      </c>
-      <c r="AL33" t="inlineStr">
-        <is>
-          <t>Traffic Signal</t>
-        </is>
-      </c>
-    </row>
-    <row r="34">
-      <c r="A34" t="n">
-        <v>14</v>
-      </c>
-      <c r="B34" t="inlineStr">
-        <is>
-          <t>SC2-S24</t>
-        </is>
-      </c>
-      <c r="C34" t="inlineStr">
-        <is>
-          <t>Ego vehicle approaching green traffic light</t>
-        </is>
-      </c>
-      <c r="D34" t="inlineStr">
-        <is>
-          <t>The ego vehicle is approaching a junction that is equipped with traffic light signals. The traffic signal for the ego vehicle is green or turns green. The objective of the ego vehicle is to cross the junction.</t>
-        </is>
-      </c>
-      <c r="E34" t="n">
-        <v>1</v>
-      </c>
-      <c r="F34" t="n">
-        <v>0</v>
-      </c>
-      <c r="G34" t="n">
-        <v>0</v>
-      </c>
-      <c r="H34" t="n">
-        <v>0</v>
-      </c>
-      <c r="I34" t="n">
-        <v>0</v>
-      </c>
-      <c r="J34" t="n">
-        <v>0</v>
-      </c>
-      <c r="K34" t="n">
-        <v>1</v>
-      </c>
-      <c r="L34" t="n">
-        <v>0</v>
-      </c>
-      <c r="M34" t="n">
-        <v>0</v>
-      </c>
-      <c r="N34" t="n">
-        <v>0</v>
-      </c>
-      <c r="O34" t="n">
-        <v>1</v>
-      </c>
-      <c r="P34" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q34" t="n">
-        <v>0</v>
-      </c>
-      <c r="R34" t="n">
-        <v>1</v>
-      </c>
-      <c r="S34" t="n">
-        <v>0</v>
-      </c>
-      <c r="T34" t="n">
-        <v>0</v>
-      </c>
-      <c r="U34" t="n">
-        <v>0</v>
-      </c>
-      <c r="V34" t="n">
-        <v>0</v>
-      </c>
-      <c r="W34" t="n">
-        <v>0</v>
-      </c>
-      <c r="X34" t="n">
-        <v>0</v>
-      </c>
-      <c r="Y34" t="n">
-        <v>0</v>
-      </c>
-      <c r="Z34" t="n">
-        <v>0</v>
-      </c>
-      <c r="AA34" t="n">
-        <v>0</v>
-      </c>
-      <c r="AB34" t="n">
-        <v>0</v>
-      </c>
-      <c r="AC34" t="n">
-        <v>0</v>
-      </c>
-      <c r="AD34" t="n">
-        <v>0</v>
-      </c>
-      <c r="AE34" t="n">
-        <v>0</v>
-      </c>
-      <c r="AF34" t="n">
-        <v>0</v>
-      </c>
-      <c r="AG34" t="n">
-        <v>1</v>
-      </c>
-      <c r="AH34" t="n">
-        <v>0</v>
-      </c>
-      <c r="AI34" t="n">
-        <v>0</v>
-      </c>
-      <c r="AJ34" t="inlineStr">
-        <is>
-          <t>sc24.png</t>
-        </is>
-      </c>
-      <c r="AK34" t="inlineStr">
-        <is>
-          <t>Singapore</t>
-        </is>
-      </c>
-      <c r="AL34" t="inlineStr">
-        <is>
-          <t>Traffic Signal</t>
-        </is>
-      </c>
-    </row>
-    <row r="35">
-      <c r="A35" t="n">
-        <v>15</v>
-      </c>
-      <c r="B35" t="inlineStr">
-        <is>
-          <t>SC2-S25</t>
-        </is>
-      </c>
-      <c r="C35" t="inlineStr">
-        <is>
-          <t xml:space="preserve"> Ego vehicle approaching amber traffic light</t>
-        </is>
-      </c>
-      <c r="D35" t="inlineStr">
-        <is>
-          <t>The ego vehicle is approaching a junction that is equipped with traffic light signals. The traffic signal for the ego vehicle is amber or turns amber. The objective of the ego vehicle is to cross the junction.</t>
-        </is>
-      </c>
-      <c r="E35" t="n">
-        <v>1</v>
-      </c>
-      <c r="F35" t="n">
-        <v>0</v>
-      </c>
-      <c r="G35" t="n">
-        <v>0</v>
-      </c>
-      <c r="H35" t="n">
-        <v>0</v>
-      </c>
-      <c r="I35" t="n">
-        <v>0</v>
-      </c>
-      <c r="J35" t="n">
-        <v>0</v>
-      </c>
-      <c r="K35" t="n">
-        <v>1</v>
-      </c>
-      <c r="L35" t="n">
-        <v>0</v>
-      </c>
-      <c r="M35" t="n">
-        <v>0</v>
-      </c>
-      <c r="N35" t="n">
-        <v>0</v>
-      </c>
-      <c r="O35" t="n">
-        <v>1</v>
-      </c>
-      <c r="P35" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q35" t="n">
-        <v>0</v>
-      </c>
-      <c r="R35" t="n">
-        <v>1</v>
-      </c>
-      <c r="S35" t="n">
-        <v>0</v>
-      </c>
-      <c r="T35" t="n">
-        <v>0</v>
-      </c>
-      <c r="U35" t="n">
-        <v>0</v>
-      </c>
-      <c r="V35" t="n">
-        <v>0</v>
-      </c>
-      <c r="W35" t="n">
-        <v>0</v>
-      </c>
-      <c r="X35" t="n">
-        <v>0</v>
-      </c>
-      <c r="Y35" t="n">
-        <v>0</v>
-      </c>
-      <c r="Z35" t="n">
-        <v>0</v>
-      </c>
-      <c r="AA35" t="n">
-        <v>0</v>
-      </c>
-      <c r="AB35" t="n">
-        <v>0</v>
-      </c>
-      <c r="AC35" t="n">
-        <v>0</v>
-      </c>
-      <c r="AD35" t="n">
-        <v>0</v>
-      </c>
-      <c r="AE35" t="n">
-        <v>0</v>
-      </c>
-      <c r="AF35" t="n">
-        <v>0</v>
-      </c>
-      <c r="AG35" t="n">
-        <v>1</v>
-      </c>
-      <c r="AH35" t="n">
-        <v>0</v>
-      </c>
-      <c r="AI35" t="n">
-        <v>0</v>
-      </c>
-      <c r="AJ35" t="inlineStr">
-        <is>
-          <t>sc25.png</t>
-        </is>
-      </c>
-      <c r="AK35" t="inlineStr">
-        <is>
-          <t>Singapore</t>
-        </is>
-      </c>
-      <c r="AL35" t="inlineStr">
-        <is>
-          <t>Traffic Signal</t>
-        </is>
-      </c>
-    </row>
-    <row r="36">
-      <c r="A36" t="n">
-        <v>16</v>
-      </c>
-      <c r="B36" t="inlineStr">
-        <is>
-          <t>SC2-S26</t>
-        </is>
-      </c>
-      <c r="C36" t="inlineStr">
-        <is>
-          <t>Vehicle running red traffic light</t>
-        </is>
-      </c>
-      <c r="D36" t="inlineStr">
-        <is>
-          <t xml:space="preserve">The ego vehicle is approaching a junction that is equipped with traffic light signals. The traffic signal for the ego vehicle is green. Another vehicle is also approaching the junction and its trajectory intersects that of the ego vehicle. The traffic signal for the other vehicle is red. However, the vehicle is running through the red light. </t>
-        </is>
-      </c>
-      <c r="E36" t="n">
-        <v>1</v>
-      </c>
-      <c r="F36" t="n">
-        <v>0</v>
-      </c>
-      <c r="G36" t="n">
-        <v>0</v>
-      </c>
-      <c r="H36" t="n">
-        <v>0</v>
-      </c>
-      <c r="I36" t="n">
-        <v>0</v>
-      </c>
-      <c r="J36" t="n">
-        <v>0</v>
-      </c>
-      <c r="K36" t="n">
-        <v>1</v>
-      </c>
-      <c r="L36" t="n">
-        <v>0</v>
-      </c>
-      <c r="M36" t="n">
-        <v>0</v>
-      </c>
-      <c r="N36" t="n">
-        <v>0</v>
-      </c>
-      <c r="O36" t="n">
-        <v>1</v>
-      </c>
-      <c r="P36" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q36" t="n">
-        <v>0</v>
-      </c>
-      <c r="R36" t="n">
-        <v>1</v>
-      </c>
-      <c r="S36" t="n">
-        <v>0</v>
-      </c>
-      <c r="T36" t="n">
-        <v>0</v>
-      </c>
-      <c r="U36" t="n">
-        <v>0</v>
-      </c>
-      <c r="V36" t="n">
-        <v>0</v>
-      </c>
-      <c r="W36" t="n">
-        <v>0</v>
-      </c>
-      <c r="X36" t="n">
-        <v>0</v>
-      </c>
-      <c r="Y36" t="n">
-        <v>0</v>
-      </c>
-      <c r="Z36" t="n">
-        <v>0</v>
-      </c>
-      <c r="AA36" t="n">
-        <v>0</v>
-      </c>
-      <c r="AB36" t="n">
-        <v>0</v>
-      </c>
-      <c r="AC36" t="n">
-        <v>0</v>
-      </c>
-      <c r="AD36" t="n">
-        <v>0</v>
-      </c>
-      <c r="AE36" t="n">
-        <v>0</v>
-      </c>
-      <c r="AF36" t="n">
-        <v>0</v>
-      </c>
-      <c r="AG36" t="n">
-        <v>1</v>
-      </c>
-      <c r="AH36" t="n">
-        <v>0</v>
-      </c>
-      <c r="AI36" t="n">
-        <v>0</v>
-      </c>
-      <c r="AJ36" t="inlineStr">
-        <is>
-          <t>sc26.png</t>
-        </is>
-      </c>
-      <c r="AK36" t="inlineStr">
-        <is>
-          <t>Singapore</t>
-        </is>
-      </c>
-      <c r="AL36" t="inlineStr">
-        <is>
-          <t>Traffic Signal</t>
-        </is>
-      </c>
-    </row>
-    <row r="37">
-      <c r="A37" t="n">
-        <v>26</v>
-      </c>
-      <c r="B37" t="inlineStr">
-        <is>
-          <t>SC2-S37</t>
-        </is>
-      </c>
-      <c r="C37" t="inlineStr">
-        <is>
-          <t>Entering a roundabout with another vehicle</t>
-        </is>
-      </c>
-      <c r="D37" t="inlineStr">
-        <is>
-          <t>The ego vehicle is approaching a round about. There is another vehicle on the roundabout or another vehicle is approaching the roundabout from another direction.</t>
-        </is>
-      </c>
-      <c r="E37" t="n">
-        <v>1</v>
-      </c>
-      <c r="F37" t="n">
-        <v>0</v>
-      </c>
-      <c r="G37" t="n">
-        <v>0</v>
-      </c>
-      <c r="H37" t="n">
-        <v>0</v>
-      </c>
-      <c r="I37" t="n">
-        <v>0</v>
-      </c>
-      <c r="J37" t="n">
-        <v>0</v>
-      </c>
-      <c r="K37" t="n">
-        <v>1</v>
-      </c>
-      <c r="L37" t="n">
-        <v>0</v>
-      </c>
-      <c r="M37" t="n">
-        <v>0</v>
-      </c>
-      <c r="N37" t="n">
-        <v>0</v>
-      </c>
-      <c r="O37" t="n">
-        <v>1</v>
-      </c>
-      <c r="P37" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q37" t="n">
-        <v>0</v>
-      </c>
-      <c r="R37" t="n">
-        <v>1</v>
-      </c>
-      <c r="S37" t="n">
-        <v>0</v>
-      </c>
-      <c r="T37" t="n">
-        <v>0</v>
-      </c>
-      <c r="U37" t="n">
-        <v>0</v>
-      </c>
-      <c r="V37" t="n">
-        <v>0</v>
-      </c>
-      <c r="W37" t="n">
-        <v>0</v>
-      </c>
-      <c r="X37" t="n">
-        <v>0</v>
-      </c>
-      <c r="Y37" t="n">
-        <v>0</v>
-      </c>
-      <c r="Z37" t="n">
-        <v>0</v>
-      </c>
-      <c r="AA37" t="n">
-        <v>0</v>
-      </c>
-      <c r="AB37" t="n">
-        <v>0</v>
-      </c>
-      <c r="AC37" t="n">
-        <v>0</v>
-      </c>
-      <c r="AD37" t="n">
-        <v>0</v>
-      </c>
-      <c r="AE37" t="n">
-        <v>0</v>
-      </c>
-      <c r="AF37" t="n">
-        <v>0</v>
-      </c>
-      <c r="AG37" t="n">
-        <v>0</v>
-      </c>
-      <c r="AH37" t="n">
-        <v>1</v>
-      </c>
-      <c r="AI37" t="n">
-        <v>0</v>
-      </c>
-      <c r="AJ37" t="inlineStr">
-        <is>
-          <t>sc37.png</t>
-        </is>
-      </c>
-      <c r="AK37" t="inlineStr">
-        <is>
-          <t>Singapore</t>
-        </is>
-      </c>
-      <c r="AL37" t="inlineStr">
         <is>
           <t>Miscellaneous</t>
         </is>

</xml_diff>